<commit_message>
Add preview URLs to import templates (#29)
</commit_message>
<xml_diff>
--- a/templates/catalog-products-import-template.xlsx
+++ b/templates/catalog-products-import-template.xlsx
@@ -84,7 +84,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -97,6 +97,7 @@
     <col min="8" max="8" style="2" width="24" customWidth="1"/>
     <col min="9" max="9" style="3" width="24" customWidth="1"/>
     <col min="10" max="10" style="3" width="20" customWidth="1"/>
+    <col min="11" max="11" style="2" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -150,9 +151,14 @@
           <t>toploader_price</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>product_preview_url</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1001"/>
+  <autoFilter ref="A1:K1001"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="0" showErrorMessage="1" errorTitle="Invalid Catalog Visibility" error="Use TRUE or FALSE." sqref="A2:A1001">
       <formula1>"TRUE,FALSE"</formula1>

</xml_diff>